<commit_message>
Office Export: neutral by default (Calibri, blue-gray, no label or byline), optional label, opt-in family art, Excel keeps its original look
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qs56CyPwtQAdyeiDNLqDfK
</commit_message>
<xml_diff>
--- a/tools/samples/Sample-Budget.xlsx
+++ b/tools/samples/Sample-Budget.xlsx
@@ -643,7 +643,7 @@
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;CPage &amp;P of &amp;N&amp;RBuzatu · Miller family</oddFooter>
+    <oddFooter>&amp;CPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -724,7 +724,7 @@
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;CPage &amp;P of &amp;N&amp;RBuzatu · Miller family</oddFooter>
+    <oddFooter>&amp;CPage &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>